<commit_message>
changed slope_vs_growth and intercept_vs_growth to slope and intercept in SectorConfig to make it pass easily to other methods
</commit_message>
<xml_diff>
--- a/tests/data/proteinAllocationModel_toymodel.xlsx
+++ b/tests/data/proteinAllocationModel_toymodel.xlsx
@@ -5,11 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="ActiveEnzymes" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="UnusedEnzyme" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Translational" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="62">
   <si>
     <t xml:space="preserve">Explanation for the test cases</t>
   </si>
@@ -138,6 +140,75 @@
   </si>
   <si>
     <t xml:space="preserve">g15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value_for_growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biomass formation reaction ID (representing growth rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ups_mu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g/g_CDW/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slope of relation between growth rate and protein concentration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ups_0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g/g_CDW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protein concentration allocated to excess enzymes at zero substrate uptake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mol_mass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g/mol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molar mass of a fictional enzyme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">substrate_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-0.004, -0.003, -0.002, -0.001]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mmol/gDW/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range of values of susbstrate uptake which are associated with linear growth regime (no fermentation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tps_mu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tps_0</t>
   </si>
 </sst>
 </file>
@@ -228,8 +299,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -255,15 +330,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:A4"/>
-  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -285,405 +360,405 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.9140625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>2000</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>1500</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="0" t="n">
+      <c r="G8" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>1500</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>2500</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="1" t="n">
         <v>2500</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G11" s="0" t="n">
+      <c r="G11" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>1122</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="0" t="n">
+      <c r="G12" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>1122</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="0" t="n">
+      <c r="G13" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>1023</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G14" s="0" t="n">
+      <c r="G14" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="1" t="n">
         <v>1023</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="0" t="n">
+      <c r="G15" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="1" t="n">
         <v>1055</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G16" s="0" t="n">
+      <c r="G16" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="0" t="n">
+      <c r="D17" s="1" t="n">
         <v>1055</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G17" s="0" t="n">
+      <c r="G17" s="1" t="n">
         <v>1000000</v>
       </c>
     </row>
@@ -694,6 +769,236 @@
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>

</xml_diff>